<commit_message>
chore(excel): standardize column headers to '输入数据 (data.py)' and '检测数据'
</commit_message>
<xml_diff>
--- a/archive/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
+++ b/archive/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
@@ -752,7 +752,7 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>数据源参数 (data.py)</t>
+          <t>输入数据 (data.py)</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="AU3" s="7" t="inlineStr">
         <is>
-          <t>评测协议</t>
+          <t>检测数据</t>
         </is>
       </c>
       <c r="AV3" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat(excel): remove redundant '评测协议 / 检测数据' column from all master tables
</commit_message>
<xml_diff>
--- a/archive/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
+++ b/archive/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV223"/>
+  <dimension ref="A1:AU223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -679,9 +679,8 @@
     <col width="10" customWidth="1" min="43" max="43"/>
     <col width="10" customWidth="1" min="44" max="44"/>
     <col width="10" customWidth="1" min="45" max="45"/>
-    <col width="34" customWidth="1" min="46" max="46"/>
-    <col width="10" customWidth="1" min="47" max="47"/>
-    <col width="65" customWidth="1" min="48" max="48"/>
+    <col width="10" customWidth="1" min="46" max="46"/>
+    <col width="65" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -926,15 +925,10 @@
       </c>
       <c r="AT3" s="7" t="inlineStr">
         <is>
-          <t>检测数据</t>
-        </is>
-      </c>
-      <c r="AU3" s="7" t="inlineStr">
-        <is>
           <t>耗时 (s)</t>
         </is>
       </c>
-      <c r="AV3" s="8" t="inlineStr">
+      <c r="AU3" s="8" t="inlineStr">
         <is>
           <t>实测现象与表现记载 (符合预期/机制归因)</t>
         </is>
@@ -1152,15 +1146,10 @@
       </c>
       <c r="AT4" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU4" s="17" t="inlineStr">
-        <is>
           <t>138.8</t>
         </is>
       </c>
-      <c r="AV4" s="19" t="inlineStr">
+      <c r="AU4" s="19" t="inlineStr">
         <is>
           <t>层数加深不解决4位加法溢出。</t>
         </is>
@@ -1378,15 +1367,10 @@
       </c>
       <c r="AT5" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU5" s="26" t="inlineStr">
-        <is>
           <t>248.0</t>
         </is>
       </c>
-      <c r="AV5" s="27" t="inlineStr">
+      <c r="AU5" s="27" t="inlineStr">
         <is>
           <t>层数加深不解决4位加法溢出。</t>
         </is>
@@ -1604,15 +1588,10 @@
       </c>
       <c r="AT6" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU6" s="17" t="inlineStr">
-        <is>
           <t>351.1</t>
         </is>
       </c>
-      <c r="AV6" s="19" t="inlineStr">
+      <c r="AU6" s="19" t="inlineStr">
         <is>
           <t>add3相变在L2→L3(63%→93%)；sub4相变在L3→L4(67%→97%)；4位加法进位受阻与层数无单调关系。</t>
         </is>
@@ -1830,15 +1809,10 @@
       </c>
       <c r="AT7" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU7" s="26" t="inlineStr">
-        <is>
           <t>485.1</t>
         </is>
       </c>
-      <c r="AV7" s="27" t="inlineStr">
+      <c r="AU7" s="27" t="inlineStr">
         <is>
           <t>add3相变在L2→L3(63%→93%)；sub4相变在L3→L4(67%→97%)；4位加法进位受阻与层数无单调关系。</t>
         </is>
@@ -2056,15 +2030,10 @@
       </c>
       <c r="AT8" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU8" s="17" t="inlineStr">
-        <is>
           <t>562.2</t>
         </is>
       </c>
-      <c r="AV8" s="19" t="inlineStr">
+      <c r="AU8" s="19" t="inlineStr">
         <is>
           <t>层数加深不解决4位加法溢出。</t>
         </is>
@@ -2282,15 +2251,10 @@
       </c>
       <c r="AT9" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU9" s="26" t="inlineStr">
-        <is>
           <t>755.1</t>
         </is>
       </c>
-      <c r="AV9" s="27" t="inlineStr">
+      <c r="AU9" s="27" t="inlineStr">
         <is>
           <t>层数加深不解决4位加法溢出。</t>
         </is>
@@ -2508,15 +2472,10 @@
       </c>
       <c r="AT10" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU10" s="17" t="inlineStr">
-        <is>
           <t>1036.2</t>
         </is>
       </c>
-      <c r="AV10" s="19" t="inlineStr">
+      <c r="AU10" s="19" t="inlineStr">
         <is>
           <t>层数加深不解决4位加法溢出。</t>
         </is>
@@ -2734,15 +2693,10 @@
       </c>
       <c r="AT11" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU11" s="26" t="inlineStr">
-        <is>
           <t>1188.0</t>
         </is>
       </c>
-      <c r="AV11" s="27" t="inlineStr">
+      <c r="AU11" s="27" t="inlineStr">
         <is>
           <t>层数加深不解决4位加法溢出。</t>
         </is>
@@ -2960,15 +2914,10 @@
       </c>
       <c r="AT12" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU12" s="17" t="inlineStr">
-        <is>
           <t>929.7</t>
         </is>
       </c>
-      <c r="AV12" s="19" t="inlineStr">
+      <c r="AU12" s="19" t="inlineStr">
         <is>
           <t>层数加深不解决4位加法溢出。</t>
         </is>
@@ -3186,15 +3135,10 @@
       </c>
       <c r="AT13" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU13" s="26" t="inlineStr">
-        <is>
           <t>1468.7</t>
         </is>
       </c>
-      <c r="AV13" s="27" t="inlineStr">
+      <c r="AU13" s="27" t="inlineStr">
         <is>
           <t>层数加深不解决4位加法溢出。</t>
         </is>
@@ -3412,15 +3356,10 @@
       </c>
       <c r="AT14" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU14" s="17" t="inlineStr">
-        <is>
           <t>51.0</t>
         </is>
       </c>
-      <c r="AV14" s="19" t="inlineStr">
+      <c r="AU14" s="19" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -3638,15 +3577,10 @@
       </c>
       <c r="AT15" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU15" s="26" t="inlineStr">
-        <is>
           <t>66.5</t>
         </is>
       </c>
-      <c r="AV15" s="27" t="inlineStr">
+      <c r="AU15" s="27" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -3864,15 +3798,10 @@
       </c>
       <c r="AT16" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU16" s="17" t="inlineStr">
-        <is>
           <t>91.0</t>
         </is>
       </c>
-      <c r="AV16" s="19" t="inlineStr">
+      <c r="AU16" s="19" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -4090,15 +4019,10 @@
       </c>
       <c r="AT17" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU17" s="26" t="inlineStr">
-        <is>
           <t>124.4</t>
         </is>
       </c>
-      <c r="AV17" s="27" t="inlineStr">
+      <c r="AU17" s="27" t="inlineStr">
         <is>
           <t>D128-D288为算术多位门槛带；D160解锁add1(97%)；D256解锁add2/3；D384 sub4达峰值87%。</t>
         </is>
@@ -4316,15 +4240,10 @@
       </c>
       <c r="AT18" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU18" s="17" t="inlineStr">
-        <is>
           <t>167.6</t>
         </is>
       </c>
-      <c r="AV18" s="19" t="inlineStr">
+      <c r="AU18" s="19" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -4542,15 +4461,10 @@
       </c>
       <c r="AT19" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU19" s="26" t="inlineStr">
-        <is>
           <t>906.8</t>
         </is>
       </c>
-      <c r="AV19" s="27" t="inlineStr">
+      <c r="AU19" s="27" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -4768,15 +4682,10 @@
       </c>
       <c r="AT20" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU20" s="17" t="inlineStr">
-        <is>
           <t>555.3</t>
         </is>
       </c>
-      <c r="AV20" s="19" t="inlineStr">
+      <c r="AU20" s="19" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -4994,15 +4903,10 @@
       </c>
       <c r="AT21" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU21" s="26" t="inlineStr">
-        <is>
           <t>841.3</t>
         </is>
       </c>
-      <c r="AV21" s="27" t="inlineStr">
+      <c r="AU21" s="27" t="inlineStr">
         <is>
           <t>D128-D288为算术多位门槛带；D160解锁add1(97%)；D256解锁add2/3；D384 sub4达峰值87%。</t>
         </is>
@@ -5220,15 +5124,10 @@
       </c>
       <c r="AT22" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU22" s="17" t="inlineStr">
-        <is>
           <t>469.8</t>
         </is>
       </c>
-      <c r="AV22" s="19" t="inlineStr">
+      <c r="AU22" s="19" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -5446,15 +5345,10 @@
       </c>
       <c r="AT23" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU23" s="26" t="inlineStr">
-        <is>
           <t>875.8</t>
         </is>
       </c>
-      <c r="AV23" s="27" t="inlineStr">
+      <c r="AU23" s="27" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -5672,15 +5566,10 @@
       </c>
       <c r="AT24" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU24" s="17" t="inlineStr">
-        <is>
           <t>762.2</t>
         </is>
       </c>
-      <c r="AV24" s="19" t="inlineStr">
+      <c r="AU24" s="19" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -5898,15 +5787,10 @@
       </c>
       <c r="AT25" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU25" s="26" t="inlineStr">
-        <is>
           <t>751.8</t>
         </is>
       </c>
-      <c r="AV25" s="27" t="inlineStr">
+      <c r="AU25" s="27" t="inlineStr">
         <is>
           <t>D128-D288为算术多位门槛带；D160解锁add1(97%)；D256解锁add2/3；D384 sub4达峰值87%。</t>
         </is>
@@ -6124,15 +6008,10 @@
       </c>
       <c r="AT26" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU26" s="17" t="inlineStr">
-        <is>
           <t>773.1</t>
         </is>
       </c>
-      <c r="AV26" s="19" t="inlineStr">
+      <c r="AU26" s="19" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -6350,15 +6229,10 @@
       </c>
       <c r="AT27" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU27" s="26" t="inlineStr">
-        <is>
           <t>714.1</t>
         </is>
       </c>
-      <c r="AV27" s="27" t="inlineStr">
+      <c r="AU27" s="27" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -6576,15 +6450,10 @@
       </c>
       <c r="AT28" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU28" s="17" t="inlineStr">
-        <is>
           <t>733.2</t>
         </is>
       </c>
-      <c r="AV28" s="19" t="inlineStr">
+      <c r="AU28" s="19" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -6802,15 +6671,10 @@
       </c>
       <c r="AT29" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU29" s="26" t="inlineStr">
-        <is>
           <t>789.2</t>
         </is>
       </c>
-      <c r="AV29" s="27" t="inlineStr">
+      <c r="AU29" s="27" t="inlineStr">
         <is>
           <t>宽度增加到288后进入稳定平台。</t>
         </is>
@@ -7028,15 +6892,10 @@
       </c>
       <c r="AT30" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU30" s="17" t="inlineStr">
-        <is>
           <t>205.5</t>
         </is>
       </c>
-      <c r="AV30" s="19" t="inlineStr">
+      <c r="AU30" s="19" t="inlineStr">
         <is>
           <t>头数对竖式特征分割存在非单调响应。</t>
         </is>
@@ -7254,15 +7113,10 @@
       </c>
       <c r="AT31" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU31" s="26" t="inlineStr">
-        <is>
           <t>216.6</t>
         </is>
       </c>
-      <c r="AV31" s="27" t="inlineStr">
+      <c r="AU31" s="27" t="inlineStr">
         <is>
           <t>头数对竖式特征分割存在非单调响应。</t>
         </is>
@@ -7480,15 +7334,10 @@
       </c>
       <c r="AT32" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU32" s="17" t="inlineStr">
-        <is>
           <t>220.1</t>
         </is>
       </c>
-      <c r="AV32" s="19" t="inlineStr">
+      <c r="AU32" s="19" t="inlineStr">
         <is>
           <t>头数对竖式特征分割存在非单调响应。</t>
         </is>
@@ -7706,15 +7555,10 @@
       </c>
       <c r="AT33" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU33" s="26" t="inlineStr">
-        <is>
           <t>254.6</t>
         </is>
       </c>
-      <c r="AV33" s="27" t="inlineStr">
+      <c r="AU33" s="27" t="inlineStr">
         <is>
           <t>【H4甜点】add2 100%, add3 70%；H5出现奇异低谷(60%)；头数非越多越好，4头最优。</t>
         </is>
@@ -7932,15 +7776,10 @@
       </c>
       <c r="AT34" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU34" s="17" t="inlineStr">
-        <is>
           <t>362.6</t>
         </is>
       </c>
-      <c r="AV34" s="19" t="inlineStr">
+      <c r="AU34" s="19" t="inlineStr">
         <is>
           <t>头数对竖式特征分割存在非单调响应。</t>
         </is>
@@ -8158,15 +7997,10 @@
       </c>
       <c r="AT35" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU35" s="26" t="inlineStr">
-        <is>
           <t>316.9</t>
         </is>
       </c>
-      <c r="AV35" s="27" t="inlineStr">
+      <c r="AU35" s="27" t="inlineStr">
         <is>
           <t>头数对竖式特征分割存在非单调响应。</t>
         </is>
@@ -8384,15 +8218,10 @@
       </c>
       <c r="AT36" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU36" s="17" t="inlineStr">
-        <is>
           <t>437.9</t>
         </is>
       </c>
-      <c r="AV36" s="19" t="inlineStr">
+      <c r="AU36" s="19" t="inlineStr">
         <is>
           <t>头数对竖式特征分割存在非单调响应。</t>
         </is>
@@ -8610,15 +8439,10 @@
       </c>
       <c r="AT37" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU37" s="26" t="inlineStr">
-        <is>
           <t>278.7</t>
         </is>
       </c>
-      <c r="AV37" s="27" t="inlineStr">
+      <c r="AU37" s="27" t="inlineStr">
         <is>
           <t>头数对竖式特征分割存在非单调响应。</t>
         </is>
@@ -8836,15 +8660,10 @@
       </c>
       <c r="AT38" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU38" s="17" t="inlineStr">
-        <is>
           <t>433.4</t>
         </is>
       </c>
-      <c r="AV38" s="19" t="inlineStr">
+      <c r="AU38" s="19" t="inlineStr">
         <is>
           <t>dp=0.0最优；Dropout破坏进位注意力模式，开启即发生单调崩溃(add4 43%→3%→0%)。</t>
         </is>
@@ -9062,15 +8881,10 @@
       </c>
       <c r="AT39" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU39" s="26" t="inlineStr">
-        <is>
           <t>480.7</t>
         </is>
       </c>
-      <c r="AV39" s="27" t="inlineStr">
+      <c r="AU39" s="27" t="inlineStr">
         <is>
           <t>Dropout过大导致模型欠拟合并丧失算术泛化。</t>
         </is>
@@ -9288,15 +9102,10 @@
       </c>
       <c r="AT40" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU40" s="17" t="inlineStr">
-        <is>
           <t>480.4</t>
         </is>
       </c>
-      <c r="AV40" s="19" t="inlineStr">
+      <c r="AU40" s="19" t="inlineStr">
         <is>
           <t>Dropout过大导致模型欠拟合并丧失算术泛化。</t>
         </is>
@@ -9514,15 +9323,10 @@
       </c>
       <c r="AT41" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU41" s="26" t="inlineStr">
-        <is>
           <t>597.9</t>
         </is>
       </c>
-      <c r="AV41" s="27" t="inlineStr">
+      <c r="AU41" s="27" t="inlineStr">
         <is>
           <t>Dropout过大导致模型欠拟合并丧失算术泛化。</t>
         </is>
@@ -9740,15 +9544,10 @@
       </c>
       <c r="AT42" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU42" s="17" t="inlineStr">
-        <is>
           <t>616.5</t>
         </is>
       </c>
-      <c r="AV42" s="19" t="inlineStr">
+      <c r="AU42" s="19" t="inlineStr">
         <is>
           <t>Dropout过大导致模型欠拟合并丧失算术泛化。</t>
         </is>
@@ -9966,15 +9765,10 @@
       </c>
       <c r="AT43" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU43" s="26" t="inlineStr">
-        <is>
           <t>137.3</t>
         </is>
       </c>
-      <c r="AV43" s="27" t="inlineStr">
+      <c r="AU43" s="27" t="inlineStr">
         <is>
           <t>线性/滑动窗口变体在长竖式计算中存在精度折损。</t>
         </is>
@@ -10192,15 +9986,10 @@
       </c>
       <c r="AT44" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU44" s="17" t="inlineStr">
-        <is>
           <t>135.3</t>
         </is>
       </c>
-      <c r="AV44" s="19" t="inlineStr">
+      <c r="AU44" s="19" t="inlineStr">
         <is>
           <t>线性/滑动窗口变体在长竖式计算中存在精度折损。</t>
         </is>
@@ -10418,15 +10207,10 @@
       </c>
       <c r="AT45" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU45" s="26" t="inlineStr">
-        <is>
           <t>128.8</t>
         </is>
       </c>
-      <c r="AV45" s="27" t="inlineStr">
+      <c r="AU45" s="27" t="inlineStr">
         <is>
           <t>线性/滑动窗口变体在长竖式计算中存在精度折损。</t>
         </is>
@@ -10644,15 +10428,10 @@
       </c>
       <c r="AT46" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU46" s="17" t="inlineStr">
-        <is>
           <t>128.6</t>
         </is>
       </c>
-      <c r="AV46" s="19" t="inlineStr">
+      <c r="AU46" s="19" t="inlineStr">
         <is>
           <t>线性/滑动窗口变体在长竖式计算中存在精度折损。</t>
         </is>
@@ -10870,15 +10649,10 @@
       </c>
       <c r="AT47" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU47" s="26" t="inlineStr">
-        <is>
           <t>127.0</t>
         </is>
       </c>
-      <c r="AV47" s="27" t="inlineStr">
+      <c r="AU47" s="27" t="inlineStr">
         <is>
           <t>线性/滑动窗口变体在长竖式计算中存在精度折损。</t>
         </is>
@@ -11096,15 +10870,10 @@
       </c>
       <c r="AT48" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU48" s="17" t="inlineStr">
-        <is>
           <t>128.3</t>
         </is>
       </c>
-      <c r="AV48" s="19" t="inlineStr">
+      <c r="AU48" s="19" t="inlineStr">
         <is>
           <t>ALiBi相对位置偏置表现突出(add1 90%)；DSA与ALiBi显著强于标准Causal。</t>
         </is>
@@ -11322,15 +11091,10 @@
       </c>
       <c r="AT49" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU49" s="26" t="inlineStr">
-        <is>
           <t>2894.1</t>
         </is>
       </c>
-      <c r="AV49" s="27" t="inlineStr">
+      <c r="AU49" s="27" t="inlineStr">
         <is>
           <t>线性/滑动窗口变体在长竖式计算中存在精度折损。</t>
         </is>
@@ -11548,15 +11312,10 @@
       </c>
       <c r="AT50" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU50" s="17" t="inlineStr">
-        <is>
           <t>123.8</t>
         </is>
       </c>
-      <c r="AV50" s="19" t="inlineStr">
+      <c r="AU50" s="19" t="inlineStr">
         <is>
           <t>专家数增加至8-16提升了细粒度分工，E8达70%峰值，E16涌现add3。</t>
         </is>
@@ -11774,15 +11533,10 @@
       </c>
       <c r="AT51" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU51" s="26" t="inlineStr">
-        <is>
           <t>146.8</t>
         </is>
       </c>
-      <c r="AV51" s="27" t="inlineStr">
+      <c r="AU51" s="27" t="inlineStr">
         <is>
           <t>专家数增加至8-16提升了细粒度分工，E8达70%峰值，E16涌现add3。</t>
         </is>
@@ -12000,15 +11754,10 @@
       </c>
       <c r="AT52" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU52" s="17" t="inlineStr">
-        <is>
           <t>182.9</t>
         </is>
       </c>
-      <c r="AV52" s="19" t="inlineStr">
+      <c r="AU52" s="19" t="inlineStr">
         <is>
           <t>专家数增加至8-16提升了细粒度分工，E8达70%峰值，E16涌现add3。</t>
         </is>
@@ -12226,15 +11975,10 @@
       </c>
       <c r="AT53" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU53" s="26" t="inlineStr">
-        <is>
           <t>238.2</t>
         </is>
       </c>
-      <c r="AV53" s="27" t="inlineStr">
+      <c r="AU53" s="27" t="inlineStr">
         <is>
           <t>专家数增加至8-16提升了细粒度分工，E8达70%峰值，E16涌现add3。</t>
         </is>
@@ -12452,15 +12196,10 @@
       </c>
       <c r="AT54" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU54" s="17" t="inlineStr">
-        <is>
           <t>373.7</t>
         </is>
       </c>
-      <c r="AV54" s="19" t="inlineStr">
+      <c r="AU54" s="19" t="inlineStr">
         <is>
           <t>专家数增加至8-16提升了细粒度分工，E8达70%峰值，E16涌现add3。</t>
         </is>
@@ -12678,15 +12417,10 @@
       </c>
       <c r="AT55" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU55" s="26" t="inlineStr">
-        <is>
           <t>238.9</t>
         </is>
       </c>
-      <c r="AV55" s="27" t="inlineStr">
+      <c r="AU55" s="27" t="inlineStr">
         <is>
           <t>topk=4显著提升梯度路由平滑度，add1达100%。</t>
         </is>
@@ -12904,15 +12638,10 @@
       </c>
       <c r="AT56" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU56" s="17" t="inlineStr">
-        <is>
           <t>286.3</t>
         </is>
       </c>
-      <c r="AV56" s="19" t="inlineStr">
+      <c r="AU56" s="19" t="inlineStr">
         <is>
           <t>topk=4显著提升梯度路由平滑度，add1达100%。</t>
         </is>
@@ -13130,15 +12859,10 @@
       </c>
       <c r="AT57" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU57" s="26" t="inlineStr">
-        <is>
           <t>383.6</t>
         </is>
       </c>
-      <c r="AV57" s="27" t="inlineStr">
+      <c r="AU57" s="27" t="inlineStr">
         <is>
           <t>topk=4显著提升梯度路由平滑度，add1达100%。</t>
         </is>
@@ -13356,15 +13080,10 @@
       </c>
       <c r="AT58" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU58" s="17" t="inlineStr">
-        <is>
           <t>303.2</t>
         </is>
       </c>
-      <c r="AV58" s="19" t="inlineStr">
+      <c r="AU58" s="19" t="inlineStr">
         <is>
           <t>aux=1.0过强导致Loss崩溃至4.19；0.01为最佳平衡点。</t>
         </is>
@@ -13582,15 +13301,10 @@
       </c>
       <c r="AT59" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU59" s="26" t="inlineStr">
-        <is>
           <t>302.1</t>
         </is>
       </c>
-      <c r="AV59" s="27" t="inlineStr">
+      <c r="AU59" s="27" t="inlineStr">
         <is>
           <t>aux=1.0过强导致Loss崩溃至4.19；0.01为最佳平衡点。</t>
         </is>
@@ -13808,15 +13522,10 @@
       </c>
       <c r="AT60" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU60" s="17" t="inlineStr">
-        <is>
           <t>299.7</t>
         </is>
       </c>
-      <c r="AV60" s="19" t="inlineStr">
+      <c r="AU60" s="19" t="inlineStr">
         <is>
           <t>aux=1.0过强导致Loss崩溃至4.19；0.01为最佳平衡点。</t>
         </is>
@@ -14034,15 +13743,10 @@
       </c>
       <c r="AT61" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU61" s="26" t="inlineStr">
-        <is>
           <t>297.7</t>
         </is>
       </c>
-      <c r="AV61" s="27" t="inlineStr">
+      <c r="AU61" s="27" t="inlineStr">
         <is>
           <t>aux=1.0过强导致Loss崩溃至4.19；0.01为最佳平衡点。</t>
         </is>
@@ -14260,15 +13964,10 @@
       </c>
       <c r="AT62" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU62" s="17" t="inlineStr">
-        <is>
           <t>295.9</t>
         </is>
       </c>
-      <c r="AV62" s="19" t="inlineStr">
+      <c r="AU62" s="19" t="inlineStr">
         <is>
           <t>aux=1.0过强导致Loss崩溃至4.19；0.01为最佳平衡点。</t>
         </is>
@@ -14486,15 +14185,10 @@
       </c>
       <c r="AT63" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU63" s="26" t="inlineStr">
-        <is>
           <t>137.5</t>
         </is>
       </c>
-      <c r="AV63" s="27" t="inlineStr">
+      <c r="AU63" s="27" t="inlineStr">
         <is>
           <t>低秩瓶颈在残差流中提供显式维度约束。</t>
         </is>
@@ -14712,15 +14406,10 @@
       </c>
       <c r="AT64" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU64" s="17" t="inlineStr">
-        <is>
           <t>137.4</t>
         </is>
       </c>
-      <c r="AV64" s="19" t="inlineStr">
+      <c r="AU64" s="19" t="inlineStr">
         <is>
           <t>【低秩增益】b=16尾部压缩促使模型聚焦关键特征，add2提升至78%(+23pp)。</t>
         </is>
@@ -14938,15 +14627,10 @@
       </c>
       <c r="AT65" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU65" s="26" t="inlineStr">
-        <is>
           <t>147.5</t>
         </is>
       </c>
-      <c r="AV65" s="27" t="inlineStr">
+      <c r="AU65" s="27" t="inlineStr">
         <is>
           <t>低秩瓶颈在残差流中提供显式维度约束。</t>
         </is>
@@ -15164,15 +14848,10 @@
       </c>
       <c r="AT66" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU66" s="17" t="inlineStr">
-        <is>
           <t>148.8</t>
         </is>
       </c>
-      <c r="AV66" s="19" t="inlineStr">
+      <c r="AU66" s="19" t="inlineStr">
         <is>
           <t>低秩瓶颈在残差流中提供显式维度约束。</t>
         </is>
@@ -15390,15 +15069,10 @@
       </c>
       <c r="AT67" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU67" s="26" t="inlineStr">
-        <is>
           <t>122.9</t>
         </is>
       </c>
-      <c r="AV67" s="27" t="inlineStr">
+      <c r="AU67" s="27" t="inlineStr">
         <is>
           <t>瓶颈位置决定压缩是在前馈阶段还是读出阶段。</t>
         </is>
@@ -15616,15 +15290,10 @@
       </c>
       <c r="AT68" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU68" s="17" t="inlineStr">
-        <is>
           <t>134.3</t>
         </is>
       </c>
-      <c r="AV68" s="19" t="inlineStr">
+      <c r="AU68" s="19" t="inlineStr">
         <is>
           <t>【架构级证实H3】末层前插入瓶颈(last_pre)导致add2降至32%，证实末层需完整通道读答案。</t>
         </is>
@@ -15842,15 +15511,10 @@
       </c>
       <c r="AT69" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU69" s="26" t="inlineStr">
-        <is>
           <t>137.0</t>
         </is>
       </c>
-      <c r="AV69" s="27" t="inlineStr">
+      <c r="AU69" s="27" t="inlineStr">
         <is>
           <t>瓶颈位置决定压缩是在前馈阶段还是读出阶段。</t>
         </is>
@@ -16068,15 +15732,10 @@
       </c>
       <c r="AT70" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU70" s="17" t="inlineStr">
-        <is>
           <t>146.1</t>
         </is>
       </c>
-      <c r="AV70" s="19" t="inlineStr">
+      <c r="AU70" s="19" t="inlineStr">
         <is>
           <t>瓶颈位置决定压缩是在前馈阶段还是读出阶段。</t>
         </is>
@@ -16294,15 +15953,10 @@
       </c>
       <c r="AT71" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU71" s="26" t="inlineStr">
-        <is>
           <t>135.7</t>
         </is>
       </c>
-      <c r="AV71" s="27" t="inlineStr">
+      <c r="AU71" s="27" t="inlineStr">
         <is>
           <t>瓶颈位置决定压缩是在前馈阶段还是读出阶段。</t>
         </is>
@@ -16520,15 +16174,10 @@
       </c>
       <c r="AT72" s="17" t="inlineStr">
         <is>
-          <t>plain_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU72" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV72" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU72" s="19" t="inlineStr">
         <is>
           <t>【无CoT多位加法恒0%】模型只能死记1位表，无法泛化到多位进位。</t>
         </is>
@@ -16746,15 +16395,10 @@
       </c>
       <c r="AT73" s="26" t="inlineStr">
         <is>
-          <t>plain_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU73" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV73" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU73" s="27" t="inlineStr">
         <is>
           <t>【无CoT多位加法恒0%】模型只能死记1位表，无法泛化到多位进位。</t>
         </is>
@@ -16972,15 +16616,10 @@
       </c>
       <c r="AT74" s="17" t="inlineStr">
         <is>
-          <t>plain_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU74" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV74" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU74" s="19" t="inlineStr">
         <is>
           <t>【无CoT多位加法恒0%】模型只能死记1位表，无法泛化到多位进位。</t>
         </is>
@@ -17198,15 +16837,10 @@
       </c>
       <c r="AT75" s="26" t="inlineStr">
         <is>
-          <t>plain_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU75" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV75" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU75" s="27" t="inlineStr">
         <is>
           <t>【无CoT多位加法恒0%】模型只能死记1位表，无法泛化到多位进位。</t>
         </is>
@@ -17424,15 +17058,10 @@
       </c>
       <c r="AT76" s="17" t="inlineStr">
         <is>
-          <t>plain_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU76" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV76" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU76" s="19" t="inlineStr">
         <is>
           <t>【无CoT多位加法恒0%】模型只能死记1位表，无法泛化到多位进位。</t>
         </is>
@@ -17650,15 +17279,10 @@
       </c>
       <c r="AT77" s="26" t="inlineStr">
         <is>
-          <t>plain_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU77" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV77" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU77" s="27" t="inlineStr">
         <is>
           <t>【无CoT多位加法恒0%】模型只能死记1位表，无法泛化到多位进位。</t>
         </is>
@@ -17876,15 +17500,10 @@
       </c>
       <c r="AT78" s="17" t="inlineStr">
         <is>
-          <t>plain_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU78" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV78" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU78" s="19" t="inlineStr">
         <is>
           <t>【无CoT多位加法恒0%】模型只能死记1位表，无法泛化到多位进位。</t>
         </is>
@@ -18102,15 +17721,10 @@
       </c>
       <c r="AT79" s="26" t="inlineStr">
         <is>
-          <t>plain_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU79" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV79" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU79" s="27" t="inlineStr">
         <is>
           <t>【无CoT多位加法恒0%】模型只能死记1位表，无法泛化到多位进位。</t>
         </is>
@@ -18328,15 +17942,10 @@
       </c>
       <c r="AT80" s="17" t="inlineStr">
         <is>
-          <t>plain_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU80" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV80" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU80" s="19" t="inlineStr">
         <is>
           <t>【无CoT多位加法恒0%】模型只能死记1位表，无法泛化到多位进位。</t>
         </is>
@@ -18554,15 +18163,10 @@
       </c>
       <c r="AT81" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU81" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV81" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU81" s="27" t="inlineStr">
         <is>
           <t>【数据形态驱动】竖式草稿纸彻底解锁多位加减法，L1D128即达67%，L4D128全面掌握。</t>
         </is>
@@ -18780,15 +18384,10 @@
       </c>
       <c r="AT82" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU82" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV82" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU82" s="19" t="inlineStr">
         <is>
           <t>【数据形态驱动】竖式草稿纸彻底解锁多位加减法，L1D128即达67%，L4D128全面掌握。</t>
         </is>
@@ -19006,15 +18605,10 @@
       </c>
       <c r="AT83" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU83" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV83" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU83" s="27" t="inlineStr">
         <is>
           <t>【数据形态驱动】竖式草稿纸彻底解锁多位加减法，L1D128即达67%，L4D128全面掌握。</t>
         </is>
@@ -19232,15 +18826,10 @@
       </c>
       <c r="AT84" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU84" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV84" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU84" s="19" t="inlineStr">
         <is>
           <t>【数据形态驱动】竖式草稿纸彻底解锁多位加减法，L1D128即达67%，L4D128全面掌握。</t>
         </is>
@@ -19458,15 +19047,10 @@
       </c>
       <c r="AT85" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU85" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV85" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU85" s="27" t="inlineStr">
         <is>
           <t>【数据形态驱动】竖式草稿纸彻底解锁多位加减法，L1D128即达67%，L4D128全面掌握。</t>
         </is>
@@ -19684,15 +19268,10 @@
       </c>
       <c r="AT86" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU86" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV86" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU86" s="19" t="inlineStr">
         <is>
           <t>【数据形态驱动】竖式草稿纸彻底解锁多位加减法，L1D128即达67%，L4D128全面掌握。</t>
         </is>
@@ -19910,15 +19489,10 @@
       </c>
       <c r="AT87" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU87" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV87" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU87" s="27" t="inlineStr">
         <is>
           <t>【数据形态驱动】竖式草稿纸彻底解锁多位加减法，L1D128即达67%，L4D128全面掌握。</t>
         </is>
@@ -20136,15 +19710,10 @@
       </c>
       <c r="AT88" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU88" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV88" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU88" s="19" t="inlineStr">
         <is>
           <t>【数据形态驱动】竖式草稿纸彻底解锁多位加减法，L1D128即达67%，L4D128全面掌握。</t>
         </is>
@@ -20362,15 +19931,10 @@
       </c>
       <c r="AT89" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU89" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV89" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU89" s="27" t="inlineStr">
         <is>
           <t>【数据形态驱动】竖式草稿纸彻底解锁多位加减法，L1D128即达67%，L4D128全面掌握。</t>
         </is>
@@ -20588,15 +20152,10 @@
       </c>
       <c r="AT90" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU90" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV90" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU90" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -20814,15 +20373,10 @@
       </c>
       <c r="AT91" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU91" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV91" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU91" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -21040,15 +20594,10 @@
       </c>
       <c r="AT92" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU92" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV92" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU92" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -21266,15 +20815,10 @@
       </c>
       <c r="AT93" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU93" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV93" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU93" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -21492,15 +21036,10 @@
       </c>
       <c r="AT94" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU94" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV94" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU94" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -21718,15 +21257,10 @@
       </c>
       <c r="AT95" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU95" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV95" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU95" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -21944,15 +21478,10 @@
       </c>
       <c r="AT96" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU96" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV96" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU96" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -22170,15 +21699,10 @@
       </c>
       <c r="AT97" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU97" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV97" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU97" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -22396,15 +21920,10 @@
       </c>
       <c r="AT98" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU98" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV98" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU98" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -22622,15 +22141,10 @@
       </c>
       <c r="AT99" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU99" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV99" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU99" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -22848,15 +22362,10 @@
       </c>
       <c r="AT100" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU100" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV100" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU100" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -23074,15 +22583,10 @@
       </c>
       <c r="AT101" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU101" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV101" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU101" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -23300,15 +22804,10 @@
       </c>
       <c r="AT102" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU102" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV102" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU102" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -23526,15 +23025,10 @@
       </c>
       <c r="AT103" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU103" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV103" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU103" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -23752,15 +23246,10 @@
       </c>
       <c r="AT104" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU104" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV104" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU104" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -23978,15 +23467,10 @@
       </c>
       <c r="AT105" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU105" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV105" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU105" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -24204,15 +23688,10 @@
       </c>
       <c r="AT106" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU106" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV106" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU106" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -24430,15 +23909,10 @@
       </c>
       <c r="AT107" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU107" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV107" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU107" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -24656,15 +24130,10 @@
       </c>
       <c r="AT108" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU108" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV108" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU108" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -24882,15 +24351,10 @@
       </c>
       <c r="AT109" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU109" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV109" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU109" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -25108,15 +24572,10 @@
       </c>
       <c r="AT110" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU110" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV110" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU110" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -25334,15 +24793,10 @@
       </c>
       <c r="AT111" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU111" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV111" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU111" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -25560,15 +25014,10 @@
       </c>
       <c r="AT112" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU112" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV112" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU112" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -25786,15 +25235,10 @@
       </c>
       <c r="AT113" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU113" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV113" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU113" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -26012,15 +25456,10 @@
       </c>
       <c r="AT114" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU114" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV114" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU114" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -26238,15 +25677,10 @@
       </c>
       <c r="AT115" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU115" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV115" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU115" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -26464,15 +25898,10 @@
       </c>
       <c r="AT116" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU116" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV116" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU116" s="19" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -26690,15 +26119,10 @@
       </c>
       <c r="AT117" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU117" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV117" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU117" s="27" t="inlineStr">
         <is>
           <t>续训降低Loss并解锁sub4/add3；但add4始终≤0.47不动，4位加法进位瓶颈非步数不足所致。</t>
         </is>
@@ -26916,15 +26340,10 @@
       </c>
       <c r="AT118" s="17" t="inlineStr">
         <is>
-          <t>selfplay_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU118" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV118" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU118" s="19" t="inlineStr">
         <is>
           <t>【Naive作弊】只出1位题(8+8=16)，坍缩到单点。</t>
         </is>
@@ -27142,15 +26561,10 @@
       </c>
       <c r="AT119" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU119" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV119" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU119" s="27" t="inlineStr">
         <is>
           <t>锚定杜绝1位作弊，但停在3位(882-22)依旧模式坍缩1/60。</t>
         </is>
@@ -27368,15 +26782,10 @@
       </c>
       <c r="AT120" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU120" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV120" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU120" s="19" t="inlineStr">
         <is>
           <t>记忆惩罚开始生效，唯一式由1增至4。</t>
         </is>
@@ -27594,15 +27003,10 @@
       </c>
       <c r="AT121" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU121" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV121" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU121" s="27" t="inlineStr">
         <is>
           <t>唯一式升至8/60，答案正确率保持95%。</t>
         </is>
@@ -27820,15 +27224,10 @@
       </c>
       <c r="AT122" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU122" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV122" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU122" s="19" t="inlineStr">
         <is>
           <t>【破坍缩甜点】40/60唯一算式 + 98.3%答案正确率，出题均值3.8位。</t>
         </is>
@@ -28046,15 +27445,10 @@
       </c>
       <c r="AT123" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU123" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV123" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU123" s="27" t="inlineStr">
         <is>
           <t>惩罚过重导致模型瞎出题，答案正确率崩跌至42%。</t>
         </is>
@@ -28272,15 +27666,10 @@
       </c>
       <c r="AT124" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU124" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV124" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU124" s="19" t="inlineStr">
         <is>
           <t>LRU遗忘窗口解决长训记忆库饱和，保持稳态多样性与高正确率。</t>
         </is>
@@ -28498,15 +27887,10 @@
       </c>
       <c r="AT125" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU125" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV125" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU125" s="27" t="inlineStr">
         <is>
           <t>坍缩到882-22=860，正确率100%。</t>
         </is>
@@ -28724,15 +28108,10 @@
       </c>
       <c r="AT126" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU126" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV126" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU126" s="19" t="inlineStr">
         <is>
           <t>【策略走捷径】坍缩到错式9999-11=91981，答案正确率崩为0%。</t>
         </is>
@@ -28950,15 +28329,10 @@
       </c>
       <c r="AT127" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU127" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV127" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU127" s="27" t="inlineStr">
         <is>
           <t>GRPO组内相对优势极其稳定，4位加法提升5pp且减法无回退。</t>
         </is>
@@ -29176,15 +28550,10 @@
       </c>
       <c r="AT128" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU128" s="17" t="inlineStr">
-        <is>
           <t>173.3</t>
         </is>
       </c>
-      <c r="AV128" s="19" t="inlineStr">
+      <c r="AU128" s="19" t="inlineStr">
         <is>
           <t>【符合预期/低秩欠拟合】r=1参数量仅占15.1%，低位减法出现轻度遗忘(sub1 40%)，4位加法保持46.7%不变。</t>
         </is>
@@ -29402,15 +28771,10 @@
       </c>
       <c r="AT129" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU129" s="26" t="inlineStr">
-        <is>
           <t>173.2</t>
         </is>
       </c>
-      <c r="AV129" s="27" t="inlineStr">
+      <c r="AU129" s="27" t="inlineStr">
         <is>
           <t>【符合预期/容量回升】r=2减法能力显著回暖(sub1 80%)，高位加法保持100%。</t>
         </is>
@@ -29628,15 +28992,10 @@
       </c>
       <c r="AT130" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU130" s="17" t="inlineStr">
-        <is>
           <t>174.1</t>
         </is>
       </c>
-      <c r="AV130" s="19" t="inlineStr">
+      <c r="AU130" s="19" t="inlineStr">
         <is>
           <t>【符合预期/黄金防遗忘点】r=4仅需17.4%参数即可在全4位微调下完整保底1-3位能力，兼具高算力效率。</t>
         </is>
@@ -29854,15 +29213,10 @@
       </c>
       <c r="AT131" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU131" s="26" t="inlineStr">
-        <is>
           <t>180.2</t>
         </is>
       </c>
-      <c r="AV131" s="27" t="inlineStr">
+      <c r="AU131" s="27" t="inlineStr">
         <is>
           <t>【符合预期/全量级复现】r=16性能追平全参数微调，1-3位全面恢复至100%。</t>
         </is>
@@ -30080,15 +29434,10 @@
       </c>
       <c r="AT132" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU132" s="17" t="inlineStr">
-        <is>
           <t>201.5</t>
         </is>
       </c>
-      <c r="AV132" s="19" t="inlineStr">
+      <c r="AU132" s="19" t="inlineStr">
         <is>
           <t>【超预期证实机制/容量饱和】即便是r=64消耗63%参数，add4依然严丝合缝卡在46.7%，证实微调无法超越预训练基座表征上限。</t>
         </is>
@@ -30306,15 +29655,10 @@
       </c>
       <c r="AT133" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU133" s="26" t="inlineStr">
-        <is>
           <t>895.1</t>
         </is>
       </c>
-      <c r="AV133" s="27" t="inlineStr">
+      <c r="AU133" s="27" t="inlineStr">
         <is>
           <t>【超预期发现/隐式进位上限】仅列和式(da+db=s)无显式进位，前2位依然达100%，但4位加减断崖崩跌至13-20%，证实长程级联必须显式草稿。</t>
         </is>
@@ -30532,15 +29876,10 @@
       </c>
       <c r="AT134" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU134" s="17" t="inlineStr">
-        <is>
           <t>900.5</t>
         </is>
       </c>
-      <c r="AV134" s="19" t="inlineStr">
+      <c r="AU134" s="19" t="inlineStr">
         <is>
           <t>【符合预期】包含进位项的全竖式列，add3达60%，格式复杂度略微增加注意力解析开销。</t>
         </is>
@@ -30758,15 +30097,10 @@
       </c>
       <c r="AT135" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU135" s="26" t="inlineStr">
-        <is>
           <t>910.2</t>
         </is>
       </c>
-      <c r="AV135" s="27" t="inlineStr">
+      <c r="AU135" s="27" t="inlineStr">
         <is>
           <t>【符合预期/基线表现】标准逐位进借位草稿纸，4位减法达46.7%，高位算术表征最平稳。</t>
         </is>
@@ -30984,15 +30318,10 @@
       </c>
       <c r="AT136" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU136" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV136" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU136" s="19" t="inlineStr">
         <is>
           <t>【符合预期】高位样本不足导致高位算术未解锁。</t>
         </is>
@@ -31210,15 +30539,10 @@
       </c>
       <c r="AT137" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU137" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV137" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU137" s="27" t="inlineStr">
         <is>
           <t>【符合预期】中等偏置过度区间。</t>
         </is>
@@ -31436,15 +30760,10 @@
       </c>
       <c r="AT138" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU138" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV138" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU138" s="19" t="inlineStr">
         <is>
           <t>【符合预期/黄金配比】2000步下展现出最佳的双位平衡收敛。</t>
         </is>
@@ -31662,15 +30981,10 @@
       </c>
       <c r="AT139" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU139" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV139" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU139" s="27" t="inlineStr">
         <is>
           <t>【符合预期】高位偏置过重影响基础数字对齐。</t>
         </is>
@@ -31888,15 +31202,10 @@
       </c>
       <c r="AT140" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU140" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV140" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU140" s="19" t="inlineStr">
         <is>
           <t>【超预期证实灾难性遗忘】100%全4位导致1位加减法(add1/sub1)彻底崩溃为0.0%！</t>
         </is>
@@ -32114,15 +31423,10 @@
       </c>
       <c r="AT141" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU141" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV141" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU141" s="27" t="inlineStr">
         <is>
           <t>【符合预期】极度偏向短题，1位加减法准确率高。</t>
         </is>
@@ -32340,15 +31644,10 @@
       </c>
       <c r="AT142" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU142" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV142" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU142" s="19" t="inlineStr">
         <is>
           <t>【符合预期】平滑过渡，解锁add2至10%。</t>
         </is>
@@ -32566,15 +31865,10 @@
       </c>
       <c r="AT143" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU143" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV143" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU143" s="27" t="inlineStr">
         <is>
           <t>【符合预期】标准衰减配置。</t>
         </is>
@@ -32792,15 +32086,10 @@
       </c>
       <c r="AT144" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU144" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV144" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU144" s="19" t="inlineStr">
         <is>
           <t>【符合预期】长题占比上升造成早期欠拟合。</t>
         </is>
@@ -33018,15 +32307,10 @@
       </c>
       <c r="AT145" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU145" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV145" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU145" s="27" t="inlineStr">
         <is>
           <t>【符合预期】均匀采样下长题分布空间过大，收敛显著拖慢。</t>
         </is>
@@ -33244,15 +32528,10 @@
       </c>
       <c r="AT146" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU146" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV146" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU146" s="19" t="inlineStr">
         <is>
           <t>【符合预期】从2位起衰减，短题极为集中。</t>
         </is>
@@ -33470,15 +32749,10 @@
       </c>
       <c r="AT147" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU147" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV147" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU147" s="27" t="inlineStr">
         <is>
           <t>【符合预期/标准基准】1-2位全枚举基底，3位以上平滑稀疏。</t>
         </is>
@@ -33696,15 +32970,10 @@
       </c>
       <c r="AT148" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU148" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV148" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU148" s="19" t="inlineStr">
         <is>
           <t>【符合预期】4位才衰减导致3位组合爆炸，早期收敛落后。</t>
         </is>
@@ -33922,15 +33191,10 @@
       </c>
       <c r="AT149" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU149" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV149" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU149" s="27" t="inlineStr">
         <is>
           <t>【符合预期】纯紧凑格式，缺少空格分隔导致token边界对齐较慢。</t>
         </is>
@@ -34148,15 +33412,10 @@
       </c>
       <c r="AT150" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU150" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV150" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU150" s="19" t="inlineStr">
         <is>
           <t>【符合预期】轻度空格扰动，模型具备适应力。</t>
         </is>
@@ -34374,15 +33633,10 @@
       </c>
       <c r="AT151" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU151" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV151" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU151" s="27" t="inlineStr">
         <is>
           <t>【符合预期】损失与准确率平稳。</t>
         </is>
@@ -34600,15 +33854,10 @@
       </c>
       <c r="AT152" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU152" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV152" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU152" s="19" t="inlineStr">
         <is>
           <t>【符合预期】0..3随机空格扰动下模型保持鲁棒。</t>
         </is>
@@ -34826,15 +34075,10 @@
       </c>
       <c r="AT153" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU153" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV153" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU153" s="27" t="inlineStr">
         <is>
           <t>【符合预期/单样本最优】单题单行消除跨样本因果干扰，高位加减法大幅领先打包模式。</t>
         </is>
@@ -35052,15 +34296,10 @@
       </c>
       <c r="AT154" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU154" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV154" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU154" s="19" t="inlineStr">
         <is>
           <t>【符合预期】小窗口打包，4位加法出现显著退化(30%→3.3%)。</t>
         </is>
@@ -35278,15 +34517,10 @@
       </c>
       <c r="AT155" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU155" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV155" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU155" s="27" t="inlineStr">
         <is>
           <t>【符合预期】跨序列注意力混杂加剧，多位加法降至10%。</t>
         </is>
@@ -35504,15 +34738,10 @@
       </c>
       <c r="AT156" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU156" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV156" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU156" s="19" t="inlineStr">
         <is>
           <t>【符合预期】长窗口全量拼接导致小模型信噪比严重不足。</t>
         </is>
@@ -35730,15 +34959,10 @@
       </c>
       <c r="AT157" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU157" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV157" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU157" s="27" t="inlineStr">
         <is>
           <t>【符合预期/基线标配】余弦平滑退火，梯度最稳定。</t>
         </is>
@@ -35956,15 +35180,10 @@
       </c>
       <c r="AT158" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU158" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV158" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU158" s="19" t="inlineStr">
         <is>
           <t>【符合预期】线性衰减末期步长偏大，略逊于余弦。</t>
         </is>
@@ -36182,15 +35401,10 @@
       </c>
       <c r="AT159" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU159" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV159" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU159" s="27" t="inlineStr">
         <is>
           <t>【符合预期】无预热余弦退火，初期收敛略快但抗冲击性弱。</t>
         </is>
@@ -36408,15 +35622,10 @@
       </c>
       <c r="AT160" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU160" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV160" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU160" s="19" t="inlineStr">
         <is>
           <t>【符合预期】纯线性调度，表现平稳。</t>
         </is>
@@ -36634,15 +35843,10 @@
       </c>
       <c r="AT161" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU161" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV161" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU161" s="27" t="inlineStr">
         <is>
           <t>【符合预期】常数学习率末期无法精细收敛，损失最高。</t>
         </is>
@@ -36860,15 +36064,10 @@
       </c>
       <c r="AT162" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU162" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV162" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU162" s="19" t="inlineStr">
         <is>
           <t>【符合预期】标准动量组合。</t>
         </is>
@@ -37086,15 +36285,10 @@
       </c>
       <c r="AT163" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU163" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV163" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU163" s="27" t="inlineStr">
         <is>
           <t>【符合预期】过渡档位。</t>
         </is>
@@ -37312,15 +36506,10 @@
       </c>
       <c r="AT164" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU164" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV164" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU164" s="19" t="inlineStr">
         <is>
           <t>【符合预期】稍大二阶动量，损失降至0.462。</t>
         </is>
@@ -37538,15 +36727,10 @@
       </c>
       <c r="AT165" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU165" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV165" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU165" s="27" t="inlineStr">
         <is>
           <t>【符合预期】PyTorch默认，表现平稳。</t>
         </is>
@@ -37764,15 +36948,10 @@
       </c>
       <c r="AT166" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU166" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV166" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU166" s="19" t="inlineStr">
         <is>
           <t>【符合预期】一阶动量0.95下平滑度高。</t>
         </is>
@@ -37990,15 +37169,10 @@
       </c>
       <c r="AT167" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU167" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV167" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU167" s="27" t="inlineStr">
         <is>
           <t>【符合预期】强裁剪未造成负面影响。</t>
         </is>
@@ -38216,15 +37390,10 @@
       </c>
       <c r="AT168" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU168" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV168" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU168" s="19" t="inlineStr">
         <is>
           <t>【符合预期/标准基线】裁剪阈值1.0稳定收敛。</t>
         </is>
@@ -38442,15 +37611,10 @@
       </c>
       <c r="AT169" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU169" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV169" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU169" s="27" t="inlineStr">
         <is>
           <t>【符合预期】弱敏感。</t>
         </is>
@@ -38668,15 +37832,10 @@
       </c>
       <c r="AT170" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU170" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV170" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU170" s="19" t="inlineStr">
         <is>
           <t>【符合预期】梯度极少超过1.0，高阈值表现一致。</t>
         </is>
@@ -38894,15 +38053,10 @@
       </c>
       <c r="AT171" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU171" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV171" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU171" s="27" t="inlineStr">
         <is>
           <t>【符合预期】收敛平稳但速度略慢。</t>
         </is>
@@ -39120,15 +38274,10 @@
       </c>
       <c r="AT172" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU172" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV172" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU172" s="19" t="inlineStr">
         <is>
           <t>【符合预期】接近最佳区域。</t>
         </is>
@@ -39346,15 +38495,10 @@
       </c>
       <c r="AT173" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU173" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV173" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU173" s="27" t="inlineStr">
         <is>
           <t>【符合预期/绝对甜点】兼具收敛速度与解题精度。</t>
         </is>
@@ -39572,15 +38716,10 @@
       </c>
       <c r="AT174" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU174" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV174" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU174" s="19" t="inlineStr">
         <is>
           <t>【符合预期】高位略有扰动但可用。</t>
         </is>
@@ -39798,15 +38937,10 @@
       </c>
       <c r="AT175" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU175" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV175" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU175" s="27" t="inlineStr">
         <is>
           <t>【符合预期】学习率偏大引起局部跳跃。</t>
         </is>
@@ -40024,15 +39158,10 @@
       </c>
       <c r="AT176" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU176" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV176" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU176" s="19" t="inlineStr">
         <is>
           <t>【符合预期】剧烈振荡，精度崩塌。</t>
         </is>
@@ -40250,15 +39379,10 @@
       </c>
       <c r="AT177" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU177" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV177" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU177" s="27" t="inlineStr">
         <is>
           <t>【符合预期】完全发散。</t>
         </is>
@@ -40476,15 +39600,10 @@
       </c>
       <c r="AT178" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU178" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV178" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU178" s="19" t="inlineStr">
         <is>
           <t>【符合预期】无权重衰减，缺乏范数收缩。</t>
         </is>
@@ -40702,15 +39821,10 @@
       </c>
       <c r="AT179" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU179" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV179" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU179" s="27" t="inlineStr">
         <is>
           <t>【符合预期】轻度正则化。</t>
         </is>
@@ -40928,15 +40042,10 @@
       </c>
       <c r="AT180" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU180" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV180" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU180" s="19" t="inlineStr">
         <is>
           <t>【符合预期/最佳正则点】有效约束嵌入与注意力和。</t>
         </is>
@@ -41154,15 +40263,10 @@
       </c>
       <c r="AT181" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU181" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV181" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU181" s="27" t="inlineStr">
         <is>
           <t>【符合预期】衰减过大造成欠拟合。</t>
         </is>
@@ -41380,15 +40484,10 @@
       </c>
       <c r="AT182" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU182" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV182" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU182" s="19" t="inlineStr">
         <is>
           <t>【符合预期】256长度对单题CoT完全足够。</t>
         </is>
@@ -41606,15 +40705,10 @@
       </c>
       <c r="AT183" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU183" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV183" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU183" s="27" t="inlineStr">
         <is>
           <t>【符合预期】表现一致。</t>
         </is>
@@ -41832,15 +40926,10 @@
       </c>
       <c r="AT184" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU184" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV184" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU184" s="19" t="inlineStr">
         <is>
           <t>【符合预期/统计稳健】seed 0基线。</t>
         </is>
@@ -42058,15 +41147,10 @@
       </c>
       <c r="AT185" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU185" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV185" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU185" s="27" t="inlineStr">
         <is>
           <t>【符合预期/统计稳健】seed 1损失与结构高度一致。</t>
         </is>
@@ -42284,15 +41368,10 @@
       </c>
       <c r="AT186" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU186" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV186" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU186" s="19" t="inlineStr">
         <is>
           <t>【符合预期/统计稳健】seed 42复现，波动小于3%。</t>
         </is>
@@ -42510,15 +41589,10 @@
       </c>
       <c r="AT187" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4 + eval=5..7)</t>
-        </is>
-      </c>
-      <c r="AU187" s="26" t="inlineStr">
-        <is>
           <t>487.8</t>
         </is>
       </c>
-      <c r="AV187" s="27" t="inlineStr">
+      <c r="AU187" s="27" t="inlineStr">
         <is>
           <t>【重大反直觉证伪/外推瓶颈不在位置编码】分布内表现优异(add4 46.7%)，但外推5/6/7位准确率全部为0.0%！原本假设相对位置能泛化，实测证伪：算术外推失败源于自回归草稿纸模板未泛化为状态机。</t>
         </is>
@@ -42736,15 +41810,10 @@
       </c>
       <c r="AT188" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU188" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV188" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU188" s="19" t="inlineStr">
         <is>
           <t>【符合预期】中等遗忘窗口，出题保持多样性(52/60唯一)，均值2.98位。</t>
         </is>
@@ -42962,15 +42031,10 @@
       </c>
       <c r="AT189" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU189" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV189" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU189" s="27" t="inlineStr">
         <is>
           <t>【超预期提升】超大滑动窗口阻断长期重复，多样性跃升至57/60。</t>
         </is>
@@ -43188,15 +42252,10 @@
       </c>
       <c r="AT190" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU190" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV190" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU190" s="19" t="inlineStr">
         <is>
           <t>【符合预期】动态课程引导避免单点坍缩，出题均值2.45位。</t>
         </is>
@@ -43414,15 +42473,10 @@
       </c>
       <c r="AT191" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU191" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV191" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU191" s="27" t="inlineStr">
         <is>
           <t>【符合预期】强制抛弃1位题，保持33/60多样性。</t>
         </is>
@@ -43640,15 +42694,10 @@
       </c>
       <c r="AT192" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU192" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV192" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU192" s="19" t="inlineStr">
         <is>
           <t>【超预期/黄金学习率】极其平缓的策略更新，达成59/60接近全散开多样性与高正确率。</t>
         </is>
@@ -43866,15 +42915,10 @@
       </c>
       <c r="AT193" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU193" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV193" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU193" s="27" t="inlineStr">
         <is>
           <t>【符合预期】略大步长引发局部坍缩至4位单题。</t>
         </is>
@@ -44092,15 +43136,10 @@
       </c>
       <c r="AT194" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU194" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV194" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU194" s="19" t="inlineStr">
         <is>
           <t>【符合预期/策略漂移】出题完全散开(57/60)，但解题能力被过大梯度冲垮。</t>
         </is>
@@ -44318,15 +43357,10 @@
       </c>
       <c r="AT195" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU195" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV195" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU195" s="27" t="inlineStr">
         <is>
           <t>【符合预期】记忆按0.9衰减，维持在4位题带。</t>
         </is>
@@ -44544,15 +43578,10 @@
       </c>
       <c r="AT196" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU196" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV196" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU196" s="19" t="inlineStr">
         <is>
           <t>【符合预期】持续约束生成空间。</t>
         </is>
@@ -44770,15 +43799,10 @@
       </c>
       <c r="AT197" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU197" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV197" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU197" s="27" t="inlineStr">
         <is>
           <t>【符合预期】给错式低分无法阻止单点坍缩。</t>
         </is>
@@ -44996,15 +44020,10 @@
       </c>
       <c r="AT198" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU198" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV198" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU198" s="19" t="inlineStr">
         <is>
           <t>【符合预期】双错给分引发策略退化。</t>
         </is>
@@ -45222,15 +44241,10 @@
       </c>
       <c r="AT199" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU199" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV199" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU199" s="27" t="inlineStr">
         <is>
           <t>【符合预期】正确不加奖导致探索停滞。</t>
         </is>
@@ -45448,15 +44462,10 @@
       </c>
       <c r="AT200" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4, lsd=True)</t>
-        </is>
-      </c>
-      <c r="AU200" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV200" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU200" s="19" t="inlineStr">
         <is>
           <t>【超预期突破/破除寻址瓶颈】逆序目标对齐 LSD 实测 add1-3=100%/100%/95%、add4=45%(sub4=100%),相对同架构正向答案的 add4 基线(约35-45%)持平未跃升,但 sub4 达 100% 说明低位优先目标完整消除了减法方向的长程反向寻址开销。加法 add4 未突破 80% 的假设落空,归因:加法高位进位累加仍需跨列前向传播,反转答案只消除了输出端寻址,未消除输入端进位链的注意力带宽瓶颈。</t>
         </is>
@@ -45674,15 +44683,10 @@
       </c>
       <c r="AT201" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4, lsd=True)</t>
-        </is>
-      </c>
-      <c r="AU201" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV201" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU201" s="27" t="inlineStr">
         <is>
           <t>【反直觉证伪/轻量级跨越失败】L2·D64 加 LSD 逆序目标实测 add1=35%、add2-4=0%(loss 0.372),并未如假设解锁 3 位进位。归因:16 万参数模型在 LSD 目标下丢失了列间进位耦合的表达力——反转答案把输出对齐负担转移给了更浅的网络,而 L2 前馈容量不足以同时承担进位状态记忆与反向解码。LSD 只对 L4 有效,不能替代深度。</t>
         </is>
@@ -45900,15 +44904,10 @@
       </c>
       <c r="AT202" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, carry_curriculum=True)</t>
-        </is>
-      </c>
-      <c r="AU202" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV202" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU202" s="19" t="inlineStr">
         <is>
           <t>【符合预期/进位深度课程有效】K=0..4 级联进位退火实测 add1-3=100%/95%/87.5%、add4=10%,sub4=20%。归因:按进位链深度 K 阶梯采样成功剥离了位数与级联深度的混淆,模型在 1-3 位进位链上注意力高度鲁棒;但 K=4 全雪崩仅 10%,证明最深的 4 级连续进位(9999+1 类)依然是表征极限,单靠采样分布无法突破进位累加器的饱和上限。</t>
         </is>
@@ -46126,15 +45125,10 @@
       </c>
       <c r="AT203" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, avalanche=True)</t>
-        </is>
-      </c>
-      <c r="AU203" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV203" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU203" s="27" t="inlineStr">
         <is>
           <t>【设计承压/极限饱和证伪】9999+1 类 100% 全雪崩压力测试实测 add1-4 全 0%(sub1=5%),loss 极低 0.0407。归因:训练分布被压缩为全进位雪崩的极窄流形,模型迅速记住了这一窄分布的统计规律(loss 极低),但没有任何跨分布泛化——测试集随机普通算式全错。这是典型的分布内记忆而非机制内化,证明极端饱和数据不能锻造进位引擎,反而造成过拟合窄域。</t>
         </is>
@@ -46352,15 +45346,10 @@
       </c>
       <c r="AT204" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4 + eval=5..7)</t>
-        </is>
-      </c>
-      <c r="AU204" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV204" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU204" s="19" t="inlineStr">
         <is>
           <t>【符合预期/循环递归初现】Looped-UT(单Block展开4步)实测 add1=77.5%、add2=37.5%、add4=10%,sub1=82.5%。归因:参数量削减 75% 的权重共享单层在 4 次展开后确实能承担单步状态机转移,1-2 位已学会;但 3-4 位进位链需要更深的展开时间步,4 步不足以让同一组注意力权重完成完整进位传播。验证了递归表达力存在,但受展开深度制约。</t>
         </is>
@@ -46578,15 +45567,10 @@
       </c>
       <c r="AT205" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4 + eval=5..7)</t>
-        </is>
-      </c>
-      <c r="AU205" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV205" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU205" s="27" t="inlineStr">
         <is>
           <t>【超预期突破/自适应展开增益显著】Looped-UT 展开 7 步实测 add1-4=92.5%/65%/22.5%/25%,显著优于 4 步版(add4 25% vs 10%)。归因:更深的展开为权重共享状态机提供了足够的迭代时间步,使进位能在同一组注意力权重上逐列前向传播,3-4 位进位首次被部分解锁。证明 Looped-UT 的算法递归性是真实可训练的,深度展开是解锁高阶进位的关键杠杆。</t>
         </is>
@@ -46804,15 +45788,10 @@
       </c>
       <c r="AT206" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, self_verify=True)</t>
-        </is>
-      </c>
-      <c r="AU206" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV206" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU206" s="19" t="inlineStr">
         <is>
           <t>【反直觉证伪/双向验算未增益】正反双向自验算 CoT(c 后反算 c-b=a)实测 add1=100%、add2=37.5%、add3-4=0%,loss 极低 0.121。归因:反向验算列虽然把正向进位图与反向借位图同时暴露给自注意力,但训练目标是预测完整序列,模型学会的是顺次复述两条列链,并未把验算作为纠错信号——答案列早于验算列生成,验算信息在因果注意力下对答案无反馈。双向结构未改变自回归单向性,故无法提升高位准确率。</t>
         </is>
@@ -47030,15 +46009,10 @@
       </c>
       <c r="AT207" s="26" t="inlineStr">
         <is>
-          <t>reader_eval(n=40, tamper_p=0.2)</t>
-        </is>
-      </c>
-      <c r="AU207" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV207" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU207" s="27" t="inlineStr">
         <is>
           <t>【反直觉证伪/Reader 惯性难以打破】草稿篡改自纠错 GRPO(20% 错误进位注入,纠错双倍奖励)实测最终模型 add1=72.5%、add2=32.5%(相对 SFT 基线 add1=82.5%/add2=62.5% 反而下降);训练中顺从错误率在 0.12~1.00 间剧烈波动,终值 1.00。归因:SFT 阶段建立的强『草稿照读』先验(Reader)使 GRPO 的纠错奖励信号被高方差优势估计淹没,模型在窄 CoT 流形上反复在纠错/顺从间摇摆,最终回归顺从惯性。证明仅靠奖励重塑不足以让极小 Transformer 从 Reader 跃升 Reasoner,需要架构级双向约束。</t>
         </is>
@@ -47256,15 +46230,10 @@
       </c>
       <c r="AT208" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU208" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV208" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU208" s="19" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 20步 极速收敛探针 实测 loss=2.0752, add1=0% add2=0% add3=0% add4=0%, sub1=0% sub4=0%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 20 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -47482,15 +46451,10 @@
       </c>
       <c r="AT209" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU209" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV209" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU209" s="27" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 50步 冒烟基线探针 实测 loss=1.6165, add1=2% add2=0% add3=0% add4=0%, sub1=8% sub4=0%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 50 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -47708,15 +46672,10 @@
       </c>
       <c r="AT210" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU210" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV210" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU210" s="19" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 100步 初期对齐探针 实测 loss=0.9919, add1=2% add2=0% add3=0% add4=0%, sub1=8% sub4=0%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 100 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -47934,15 +46893,10 @@
       </c>
       <c r="AT211" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU211" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV211" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU211" s="27" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 200步 早期学习探针 实测 loss=0.6842, add1=2% add2=0% add3=0% add4=0%, sub1=22% sub4=0%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 200 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -48160,15 +47114,10 @@
       </c>
       <c r="AT212" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU212" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV212" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU212" s="19" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 500步 初步收敛探针 实测 loss=0.3467, add1=20% add2=0% add3=0% add4=0%, sub1=25% sub4=0%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 500 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -48386,15 +47335,10 @@
       </c>
       <c r="AT213" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU213" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV213" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU213" s="27" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 1,000步 早期阶段基线 实测 loss=0.2241, add1=40% add2=10% add3=0% add4=0%, sub1=58% sub4=0%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 1,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -48612,15 +47556,10 @@
       </c>
       <c r="AT214" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU214" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV214" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU214" s="19" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 2,000步 半程收敛探针 实测 loss=0.1627, add1=92% add2=88% add3=48% add4=0%, sub1=100% sub4=18%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 2,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -48838,15 +47777,10 @@
       </c>
       <c r="AT215" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU215" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV215" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU215" s="27" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 4,000步 标准基线 实测 loss=0.1728, add1=98% add2=95% add3=75% add4=20%, sub1=100% sub4=38%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 4,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -49064,15 +47998,10 @@
       </c>
       <c r="AT216" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU216" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV216" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU216" s="19" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 8,000步 翻倍扩展 实测 loss=0.1713, add1=100% add2=95% add3=75% add4=30%, sub1=100% sub4=60%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 8,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -49290,15 +48219,10 @@
       </c>
       <c r="AT217" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU217" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV217" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU217" s="27" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 16,000步 长程扩展 实测 loss=0.1693, add1=100% add2=100% add3=95% add4=40%, sub1=100% sub4=88%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 16,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -49516,15 +48440,10 @@
       </c>
       <c r="AT218" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU218" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV218" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU218" s="19" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 32,000步 深度训练 实测 loss=0.1687, add1=100% add2=100% add3=95% add4=35%, sub1=100% sub4=90%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 32,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -49742,15 +48661,10 @@
       </c>
       <c r="AT219" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU219" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV219" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU219" s="27" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 64,000步 超长训练 实测 loss=0.1694, add1=100% add2=100% add3=100% add4=45%, sub1=100% sub4=95%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 64,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -49968,15 +48882,10 @@
       </c>
       <c r="AT220" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU220" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV220" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU220" s="19" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 128,000步 缩放扫描 实测 loss=0.1853, add1=100% add2=100% add3=100% add4=40%, sub1=100% sub4=92%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 128,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -50194,15 +49103,10 @@
       </c>
       <c r="AT221" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU221" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV221" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU221" s="27" t="inlineStr">
         <is>
           <t>【实测/步数扩展】L4_D128 CoT 256,000步 大算力训练 实测 loss=0.1759, add1=100% add2=100% add3=100% add4=45%, sub1=100% sub4=100%。归因:沿同一条 L4_D128 CoT 连续训练曲线在 256,000 步处采样,刻画损失下探与多位泛化边界随训练算力的边际曲线;验证算术能力随步数增长的规律。</t>
         </is>
@@ -50420,15 +49324,10 @@
       </c>
       <c r="AT222" s="17" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU222" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV222" s="19" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU222" s="19" t="inlineStr">
         <is>
           <t>【待运行 / 未跑】连续训练曲线尚未推进到 512,000 步,评测待曲线完成该步数后回填。</t>
         </is>
@@ -50646,15 +49545,10 @@
       </c>
       <c r="AT223" s="26" t="inlineStr">
         <is>
-          <t>cot_eval(n=40, digits=1..4)</t>
-        </is>
-      </c>
-      <c r="AU223" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="AV223" s="27" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="AU223" s="27" t="inlineStr">
         <is>
           <t>【待运行 / 未跑】连续训练曲线尚未推进到 1,024,000 步,评测待曲线完成该步数后回填。</t>
         </is>
@@ -50662,8 +49556,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:AV1"/>
-    <mergeCell ref="A2:AV2"/>
+    <mergeCell ref="A2:AU2"/>
+    <mergeCell ref="A1:AU1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(excel): change Add1..Sub4 headers to 算式:得分 and add Sheet 2 with 40 benchmark questions
</commit_message>
<xml_diff>
--- a/archive/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
+++ b/archive/ALL_DOCS_EXPERIMENTS_CONFIG_TO_RESULTS.xlsx
@@ -669,17 +669,17 @@
     <col width="11" customWidth="1" min="33" max="33"/>
     <col width="11" customWidth="1" min="34" max="34"/>
     <col width="11" customWidth="1" min="35" max="35"/>
-    <col width="10" customWidth="1" min="36" max="36"/>
-    <col width="10" customWidth="1" min="37" max="37"/>
-    <col width="10" customWidth="1" min="38" max="38"/>
-    <col width="10" customWidth="1" min="39" max="39"/>
-    <col width="10" customWidth="1" min="40" max="40"/>
-    <col width="10" customWidth="1" min="41" max="41"/>
-    <col width="10" customWidth="1" min="42" max="42"/>
-    <col width="10" customWidth="1" min="43" max="43"/>
-    <col width="10" customWidth="1" min="44" max="44"/>
-    <col width="10" customWidth="1" min="45" max="45"/>
-    <col width="10" customWidth="1" min="46" max="46"/>
+    <col width="17" customWidth="1" min="36" max="36"/>
+    <col width="17" customWidth="1" min="37" max="37"/>
+    <col width="17" customWidth="1" min="38" max="38"/>
+    <col width="17" customWidth="1" min="39" max="39"/>
+    <col width="17" customWidth="1" min="40" max="40"/>
+    <col width="17" customWidth="1" min="41" max="41"/>
+    <col width="17" customWidth="1" min="42" max="42"/>
+    <col width="17" customWidth="1" min="43" max="43"/>
+    <col width="12" customWidth="1" min="44" max="44"/>
+    <col width="12" customWidth="1" min="45" max="45"/>
+    <col width="12" customWidth="1" min="46" max="46"/>
     <col width="65" customWidth="1" min="47" max="47"/>
   </cols>
   <sheetData>
@@ -875,42 +875,42 @@
       </c>
       <c r="AJ3" s="7" t="inlineStr">
         <is>
-          <t>Add1 %</t>
+          <t>Add1 (算式:得分)</t>
         </is>
       </c>
       <c r="AK3" s="7" t="inlineStr">
         <is>
-          <t>Add2 %</t>
+          <t>Add2 (算式:得分)</t>
         </is>
       </c>
       <c r="AL3" s="7" t="inlineStr">
         <is>
-          <t>Add3 %</t>
+          <t>Add3 (算式:得分)</t>
         </is>
       </c>
       <c r="AM3" s="7" t="inlineStr">
         <is>
-          <t>Add4 %</t>
+          <t>Add4 (算式:得分)</t>
         </is>
       </c>
       <c r="AN3" s="7" t="inlineStr">
         <is>
-          <t>Sub1 %</t>
+          <t>Sub1 (算式:得分)</t>
         </is>
       </c>
       <c r="AO3" s="7" t="inlineStr">
         <is>
-          <t>Sub2 %</t>
+          <t>Sub2 (算式:得分)</t>
         </is>
       </c>
       <c r="AP3" s="7" t="inlineStr">
         <is>
-          <t>Sub3 %</t>
+          <t>Sub3 (算式:得分)</t>
         </is>
       </c>
       <c r="AQ3" s="7" t="inlineStr">
         <is>
-          <t>Sub4 %</t>
+          <t>Sub4 (算式:得分)</t>
         </is>
       </c>
       <c r="AR3" s="7" t="inlineStr">

</xml_diff>